<commit_message>
feat(artefacts): update vision board avec Mme Lefevre corrigée
</commit_message>
<xml_diff>
--- a/cadrage/equipe-24-vision-board-v1.0.xlsx
+++ b/cadrage/equipe-24-vision-board-v1.0.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabriel/Documents/apocalipssi-models/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabriel/Documents/code/IPSSI_APOCAL_KIT/cadrage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31C20595-53EE-384E-AE08-8DD62FBD282A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E5A874F-CDFF-5941-8F02-318B0E4B0161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="22900" windowHeight="17780" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -237,9 +237,6 @@
     <t>Nadia Hakimi</t>
   </si>
   <si>
-    <t>47 ans, enseignante BTS/Licence, prepare seule ses cours, 1h+ a creer des exercices manuellement, à l'aise bureautique, sensible à la confidentialité des contenus pédagogiques</t>
-  </si>
-  <si>
     <t>21 ans, étudiante BTS/Licence, passe les quiz générés par ses profs, veut identifier ses lacunes et réviser ses erreurs entre sessions</t>
   </si>
   <si>
@@ -400,6 +397,9 @@
   </si>
   <si>
     <t>Pour les enseignants du supérieur qui passent plus d'une heure à créer des évaluations alignées sur leur cours réel, EduTutor IA est une plateforme de génération de QCM par IA locale souveraine qui permet de transformer n'importe quel support de cours en quiz prêt à utiliser en classe en moins d'une minute, sans transfert de données hors-UE. Contrairement à Quizlet AI, Khanmigo et Leo étudiant-first, cloud américain notre produit inverse le modèle : l'enseignant dépose, l'IA évalue, la donnée reste.</t>
+  </si>
+  <si>
+    <t>42 ans, enseignante BTS Communication à Lyon, 28 étudiants sous sa responsabilité. Veut visualiser les scores de sa classe, repérer les décrocheurs et envoyer des conseils adaptés. À l'aise avec les outils numériques, non-dev. Sensible à la conformité des données.</t>
   </si>
 </sst>
 </file>
@@ -689,138 +689,138 @@
   </cellStyleXfs>
   <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1101,485 +1101,485 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
     </row>
     <row r="2" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
     </row>
     <row r="4" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
     </row>
     <row r="5" spans="1:5" ht="49.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="15"/>
-      <c r="B5" s="11" t="s">
+      <c r="A5" s="1"/>
+      <c r="B5" s="41" t="s">
         <v>62</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="15"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
+      <c r="B6" s="42"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
     </row>
     <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="70" x14ac:dyDescent="0.2">
-      <c r="A10" s="17" t="s">
+    <row r="10" spans="1:5" ht="98" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E10" s="17" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="56" x14ac:dyDescent="0.2">
-      <c r="A11" s="19" t="s">
+      <c r="E11" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B13" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
+    </row>
+    <row r="15" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+      <c r="A17" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+      <c r="A18" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="20" t="s">
-        <v>67</v>
-      </c>
-      <c r="E11" s="19" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="56" x14ac:dyDescent="0.2">
-      <c r="A12" s="17" t="s">
+      <c r="B18" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+      <c r="A19" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>68</v>
-      </c>
-      <c r="E12" s="17" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B13" s="8" t="s">
+      <c r="B19" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-    </row>
-    <row r="15" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="21" t="s">
+      <c r="D19" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="56" x14ac:dyDescent="0.2">
+      <c r="A20" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+      <c r="A21" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="B23" s="36"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="36"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="E16" s="21" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="A17" s="22" t="s">
+      <c r="B24" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="28" x14ac:dyDescent="0.2">
+      <c r="A25" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="23" t="s">
-        <v>72</v>
-      </c>
-      <c r="C17" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>77</v>
-      </c>
-      <c r="E17" s="22" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="56" x14ac:dyDescent="0.2">
-      <c r="A18" s="19" t="s">
+      <c r="B25" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="28" x14ac:dyDescent="0.2">
+      <c r="A26" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="C18" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="D18" s="20" t="s">
-        <v>78</v>
-      </c>
-      <c r="E18" s="19" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="56" x14ac:dyDescent="0.2">
-      <c r="A19" s="22" t="s">
+      <c r="B26" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="28" x14ac:dyDescent="0.2">
+      <c r="A27" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="C19" s="23" t="s">
-        <v>70</v>
-      </c>
-      <c r="D19" s="23" t="s">
-        <v>79</v>
-      </c>
-      <c r="E19" s="22" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="56" x14ac:dyDescent="0.2">
-      <c r="A20" s="19" t="s">
+      <c r="B27" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="E27" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="28" x14ac:dyDescent="0.2">
+      <c r="A28" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="C20" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="D20" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="E20" s="19" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="A21" s="22" t="s">
+      <c r="B28" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="28" x14ac:dyDescent="0.2">
+      <c r="A29" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="C21" s="23" t="s">
-        <v>71</v>
-      </c>
-      <c r="D21" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="E21" s="22" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="24" t="s">
+      <c r="B29" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="E29" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" s="37"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="37"/>
+      <c r="E31" s="37"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="B24" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="C24" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="E24" s="24" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="28" x14ac:dyDescent="0.2">
-      <c r="A25" s="25" t="s">
+      <c r="B32" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="D32" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E32" s="13" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="42" x14ac:dyDescent="0.2">
+      <c r="A33" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B25" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="C25" s="26" t="s">
-        <v>87</v>
-      </c>
-      <c r="D25" s="25" t="s">
-        <v>32</v>
-      </c>
-      <c r="E25" s="25" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="28" x14ac:dyDescent="0.2">
-      <c r="A26" s="19" t="s">
+      <c r="B33" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="28" x14ac:dyDescent="0.2">
+      <c r="A34" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B26" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="C26" s="20" t="s">
-        <v>88</v>
-      </c>
-      <c r="D26" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="E26" s="19" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="28" x14ac:dyDescent="0.2">
-      <c r="A27" s="25" t="s">
+      <c r="B34" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="28" x14ac:dyDescent="0.2">
+      <c r="A35" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="26" t="s">
-        <v>84</v>
-      </c>
-      <c r="C27" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="D27" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="E27" s="25" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="28" x14ac:dyDescent="0.2">
-      <c r="A28" s="19" t="s">
+      <c r="B35" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="28" x14ac:dyDescent="0.2">
+      <c r="A36" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B28" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="C28" s="20" t="s">
-        <v>90</v>
-      </c>
-      <c r="D28" s="19" t="s">
-        <v>94</v>
-      </c>
-      <c r="E28" s="19" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="28" x14ac:dyDescent="0.2">
-      <c r="A29" s="25" t="s">
+      <c r="B36" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C36" s="31">
+        <v>0.75</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="28" x14ac:dyDescent="0.2">
+      <c r="A37" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B29" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="C29" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="D29" s="25" t="s">
-        <v>95</v>
-      </c>
-      <c r="E29" s="25" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="B32" s="27" t="s">
-        <v>37</v>
-      </c>
-      <c r="C32" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="D32" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="E32" s="27" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="42" x14ac:dyDescent="0.2">
-      <c r="A33" s="28" t="s">
-        <v>9</v>
-      </c>
-      <c r="B33" s="29" t="s">
-        <v>96</v>
-      </c>
-      <c r="C33" s="29" t="s">
-        <v>97</v>
-      </c>
-      <c r="D33" s="28" t="s">
-        <v>98</v>
-      </c>
-      <c r="E33" s="29" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="28" x14ac:dyDescent="0.2">
-      <c r="A34" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="B34" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="C34" s="20" t="s">
-        <v>101</v>
-      </c>
-      <c r="D34" s="19" t="s">
-        <v>102</v>
-      </c>
-      <c r="E34" s="20" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="28" x14ac:dyDescent="0.2">
-      <c r="A35" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="B35" s="29" t="s">
-        <v>104</v>
-      </c>
-      <c r="C35" s="29" t="s">
-        <v>105</v>
-      </c>
-      <c r="D35" s="28" t="s">
-        <v>106</v>
-      </c>
-      <c r="E35" s="29" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="28" x14ac:dyDescent="0.2">
-      <c r="A36" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="B36" s="20" t="s">
-        <v>108</v>
-      </c>
-      <c r="C36" s="46">
-        <v>0.75</v>
-      </c>
-      <c r="D36" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="E36" s="20" t="s">
+      <c r="B37" s="15" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" ht="28" x14ac:dyDescent="0.2">
-      <c r="A37" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="B37" s="29" t="s">
+      <c r="C37" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="C37" s="29" t="s">
+      <c r="D37" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E37" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="D37" s="28" t="s">
-        <v>113</v>
-      </c>
-      <c r="E37" s="29" t="s">
-        <v>112</v>
-      </c>
     </row>
     <row r="39" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
+      <c r="B39" s="32"/>
+      <c r="C39" s="32"/>
+      <c r="D39" s="32"/>
+      <c r="E39" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A31:E31"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B6:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -1601,134 +1601,134 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="D4" s="16" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="33" t="s">
+      <c r="C5" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="28" x14ac:dyDescent="0.2">
+      <c r="A6" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="D5" s="34" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="28" x14ac:dyDescent="0.2">
-      <c r="A6" s="35" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="36" t="s">
-        <v>50</v>
-      </c>
-      <c r="C6" s="33" t="s">
+      <c r="D6" s="20" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="28" x14ac:dyDescent="0.2">
+      <c r="A7" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="D6" s="34" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="28" x14ac:dyDescent="0.2">
-      <c r="A7" s="37" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="38" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7" s="33" t="s">
+      <c r="D7" s="20" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+      <c r="A8" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="D7" s="34" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="42" x14ac:dyDescent="0.2">
-      <c r="A8" s="39" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="40" t="s">
-        <v>54</v>
-      </c>
-      <c r="C8" s="33" t="s">
+      <c r="D8" s="20" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+      <c r="A9" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="D8" s="34" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="42" x14ac:dyDescent="0.2">
-      <c r="A9" s="41" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="42" t="s">
-        <v>56</v>
-      </c>
-      <c r="C9" s="33" t="s">
+      <c r="D9" s="20" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="42" x14ac:dyDescent="0.2">
+      <c r="A10" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="D9" s="34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="42" x14ac:dyDescent="0.2">
-      <c r="A10" s="43" t="s">
-        <v>58</v>
-      </c>
-      <c r="B10" s="44" t="s">
-        <v>59</v>
-      </c>
-      <c r="C10" s="33" t="s">
+      <c r="D10" s="20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="45" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="45"/>
+      <c r="C12" s="45"/>
+      <c r="D12" s="45"/>
+    </row>
+    <row r="13" spans="1:4" ht="49.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="46" t="s">
         <v>119</v>
       </c>
-      <c r="D10" s="34" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-    </row>
-    <row r="13" spans="1:4" ht="49.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="45" t="s">
-        <v>120</v>
-      </c>
-      <c r="B13" s="45"/>
-      <c r="C13" s="45"/>
-      <c r="D13" s="45"/>
+      <c r="B13" s="46"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
feat(artefacts): update vision board avec Lea Moreau role primaire
</commit_message>
<xml_diff>
--- a/cadrage/equipe-24-vision-board-v1.0.xlsx
+++ b/cadrage/equipe-24-vision-board-v1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabriel/Documents/code/IPSSI_APOCAL_KIT/cadrage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E5A874F-CDFF-5941-8F02-318B0E4B0161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EAE3D73-BDA6-6748-B964-99A2A4C04EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="22900" windowHeight="17780" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="119">
   <si>
     <t>📋 PRODUCT VISION BOARD — SkillHub</t>
   </si>
@@ -76,12 +76,6 @@
   </si>
   <si>
     <t>2</t>
-  </si>
-  <si>
-    <t>Secondaire</t>
-  </si>
-  <si>
-    <t>Moyenne</t>
   </si>
   <si>
     <t>3</t>
@@ -782,6 +776,19 @@
     <xf numFmtId="9" fontId="4" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -798,19 +805,6 @@
     <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1101,54 +1095,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
     </row>
     <row r="2" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
     </row>
     <row r="4" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
+      <c r="B4" s="34"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="34"/>
     </row>
     <row r="5" spans="1:5" ht="49.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
-      <c r="B5" s="41" t="s">
-        <v>62</v>
-      </c>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
+      <c r="B5" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="42"/>
-      <c r="C6" s="42"/>
-      <c r="D6" s="42"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="36"/>
+      <c r="D6" s="36"/>
     </row>
     <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
+      <c r="B8" s="38"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
@@ -1172,13 +1166,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
@@ -1189,63 +1183,63 @@
         <v>12</v>
       </c>
       <c r="B11" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>66</v>
-      </c>
       <c r="E11" s="5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C12" s="3" t="s">
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B13" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+    </row>
+    <row r="15" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B13" s="34" t="s">
-        <v>68</v>
-      </c>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-    </row>
-    <row r="15" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="35" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="35"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="35"/>
+      <c r="B15" s="40"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
         <v>4</v>
       </c>
       <c r="B16" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>19</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>21</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>8</v>
@@ -1256,16 +1250,16 @@
         <v>9</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="56" x14ac:dyDescent="0.2">
@@ -1273,93 +1267,93 @@
         <v>12</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A19" s="8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="56" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="42" x14ac:dyDescent="0.2">
       <c r="A21" s="8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="36" t="s">
-        <v>26</v>
-      </c>
-      <c r="B23" s="36"/>
-      <c r="C23" s="36"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="36"/>
+      <c r="A23" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23" s="41"/>
+      <c r="C23" s="41"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="41"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="10" t="s">
         <v>4</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C24" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="28" x14ac:dyDescent="0.2">
@@ -1367,16 +1361,16 @@
         <v>9</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="28" x14ac:dyDescent="0.2">
@@ -1384,93 +1378,93 @@
         <v>12</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="28" x14ac:dyDescent="0.2">
       <c r="A27" s="11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="28" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="28" x14ac:dyDescent="0.2">
       <c r="A29" s="11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="37" t="s">
-        <v>36</v>
-      </c>
-      <c r="B31" s="37"/>
-      <c r="C31" s="37"/>
-      <c r="D31" s="37"/>
-      <c r="E31" s="37"/>
+      <c r="A31" s="42" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31" s="42"/>
+      <c r="C31" s="42"/>
+      <c r="D31" s="42"/>
+      <c r="E31" s="42"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="13" t="s">
         <v>4</v>
       </c>
       <c r="B32" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D32" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="13" t="s">
+      <c r="E32" s="13" t="s">
         <v>38</v>
-      </c>
-      <c r="D32" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="42" x14ac:dyDescent="0.2">
@@ -1478,16 +1472,16 @@
         <v>9</v>
       </c>
       <c r="B33" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="D33" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="C33" s="15" t="s">
+      <c r="E33" s="15" t="s">
         <v>96</v>
-      </c>
-      <c r="D33" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="E33" s="15" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="28" x14ac:dyDescent="0.2">
@@ -1495,91 +1489,91 @@
         <v>12</v>
       </c>
       <c r="B34" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D34" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="E34" s="6" t="s">
         <v>100</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="28" x14ac:dyDescent="0.2">
       <c r="A35" s="14" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B35" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="D35" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="C35" s="15" t="s">
+      <c r="E35" s="15" t="s">
         <v>104</v>
-      </c>
-      <c r="D35" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="E35" s="15" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="28" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C36" s="31">
         <v>0.75</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="28" x14ac:dyDescent="0.2">
       <c r="A37" s="14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B37" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="E37" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="C37" s="15" t="s">
-        <v>110</v>
-      </c>
-      <c r="D37" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="E37" s="15" t="s">
-        <v>111</v>
-      </c>
     </row>
     <row r="39" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="B39" s="32"/>
-      <c r="C39" s="32"/>
-      <c r="D39" s="32"/>
-      <c r="E39" s="32"/>
+      <c r="A39" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39" s="37"/>
+      <c r="C39" s="37"/>
+      <c r="D39" s="37"/>
+      <c r="E39" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B6:D6"/>
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A8:E8"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -1602,7 +1596,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="43" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B1" s="43"/>
       <c r="C1" s="43"/>
@@ -1610,7 +1604,7 @@
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="44" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B2" s="44"/>
       <c r="C2" s="44"/>
@@ -1621,13 +1615,13 @@
         <v>4</v>
       </c>
       <c r="B4" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="16" t="s">
         <v>45</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -1635,13 +1629,13 @@
         <v>9</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="28" x14ac:dyDescent="0.2">
@@ -1649,74 +1643,74 @@
         <v>12</v>
       </c>
       <c r="B6" s="22" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="28" x14ac:dyDescent="0.2">
       <c r="A7" s="23" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="42" x14ac:dyDescent="0.2">
       <c r="A8" s="25" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="42" x14ac:dyDescent="0.2">
       <c r="A9" s="27" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B9" s="28" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="42" x14ac:dyDescent="0.2">
       <c r="A10" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="D10" s="20" t="s">
         <v>58</v>
-      </c>
-      <c r="B10" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="D10" s="20" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="45" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B12" s="45"/>
       <c r="C12" s="45"/>
@@ -1724,7 +1718,7 @@
     </row>
     <row r="13" spans="1:4" ht="49.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="46" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B13" s="46"/>
       <c r="C13" s="46"/>

</xml_diff>